<commit_message>
Sincronización total del proyecto: Incluyendo datasets de prueba y normativas adicionales
</commit_message>
<xml_diff>
--- a/Plantilla_Auditoria_Modelo3.xlsx
+++ b/Plantilla_Auditoria_Modelo3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LL_AgenteIIBB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5EC8AD-1BDA-480E-B310-B898987F592C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C53B94E-1745-4F38-8F41-DA6814A42E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2460" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos Auditoría" sheetId="1" r:id="rId1"/>
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Cuit</t>
   </si>
@@ -217,13 +217,31 @@
     <t>Situacion_Especial</t>
   </si>
   <si>
-    <t>MO</t>
-  </si>
-  <si>
     <t>Servicios Profesionales Contables</t>
   </si>
   <si>
     <t>Profesional Recibido con título universitario y matriculado</t>
+  </si>
+  <si>
+    <t>RI</t>
+  </si>
+  <si>
+    <t>VENTA AL POR MAYOR DE PRODUCTOS FARMACÉUTICOS</t>
+  </si>
+  <si>
+    <t>No existe situación especial que se conozca</t>
+  </si>
+  <si>
+    <t>Servicios de consultoría informática</t>
+  </si>
+  <si>
+    <t>620100</t>
+  </si>
+  <si>
+    <t>Desarrollo de software y exportación de servicios a España</t>
+  </si>
+  <si>
+    <t>Empresa PyME con certificado vigente</t>
   </si>
 </sst>
 </file>
@@ -614,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="10" width="20.7109375" customWidth="1"/>
@@ -660,19 +678,80 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1000000</v>
+      </c>
+      <c r="G2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="2">
-        <v>1500000</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
+      <c r="H2">
+        <v>5</v>
       </c>
       <c r="I2">
         <v>902</v>
       </c>
       <c r="J2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>20341372659</v>
+      </c>
+      <c r="B3">
+        <v>2026</v>
+      </c>
+      <c r="C3" t="s">
         <v>12</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1500000000</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3">
+        <v>464310</v>
+      </c>
+      <c r="I3">
+        <v>902</v>
+      </c>
+      <c r="J3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>20341372659</v>
+      </c>
+      <c r="B4">
+        <v>2026</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1500000</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4">
+        <v>3.5</v>
+      </c>
+      <c r="I4">
+        <v>902</v>
+      </c>
+      <c r="J4" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>